<commit_message>
Store page hero images in the shared DAM heros folder
The homepage import now maps hero images (and the matching metadata
image) to /content/dam/nzdoc/heros/<file name> instead of a path
derived from the source URL.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,9 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>heroImages</t>
+  </si>
+  <si>
     <t>path</t>
   </si>
   <si>
@@ -43,6 +46,9 @@
     <t>["hero","feedback"]</t>
   </si>
   <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg</t>
+  </si>
+  <si>
     <t>index</t>
   </si>
   <si>
@@ -52,7 +58,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T02:02:52.120Z</t>
+    <t>2026-09-28T02:13:43.592Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -447,19 +453,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="7" customWidth="1"/>
-    <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="33" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="7" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="33" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -484,35 +491,41 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:I1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add homepage panels: typed cards, columns with content lists
- Card: Type dropdown (Short Walks / Blog) driving the layout, plus
  image, title, date, content title, link, text and optional More.
  Lint cell limit raised to 8 for the card model only.
- New Content List block: 4 content item pickers rendered as page
  teasers (title, description, image) and an optional More link.
- Columns: allow Content List in columns, decorate/load blocks nested
  in a column and style those columns as titled panels.
- Content column width 961px, 24px gap below the hero, Zilla Slab
  fonts moved to the shared font stylesheet.
- Homepage import: cards and columns parsers, section grouping in the
  cleanup transformer, More links for content lists in the report.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,6 +19,9 @@
     <t>blocks</t>
   </si>
   <si>
+    <t>contentListMore</t>
+  </si>
+  <si>
     <t>heroImages</t>
   </si>
   <si>
@@ -43,7 +46,10 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["hero","feedback"]</t>
+    <t>["hero","cards","columns","feedback"]</t>
+  </si>
+  <si>
+    <t>Featured: https://www.doc.govt.nz/footer-links/new-on-the-site/; Media releases: https://www.doc.govt.nz/news/media-releases/2026-media-releases/</t>
   </si>
   <si>
     <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg</t>
@@ -58,7 +64,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T02:13:43.592Z</t>
+    <t>2026-09-28T02:52:36.786Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -453,20 +459,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="7" customWidth="1"/>
-    <col min="6" max="6" width="10" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="33" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="2" max="2" width="39" customWidth="1"/>
+    <col min="3" max="4" width="50" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="33" customWidth="1"/>
+    <col min="10" max="10" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -494,38 +500,44 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Map homepage card images to DAM folders
The homepage import now stores Short Walks card images with the page
heroes (/content/dam/nzdoc/heros) and DOC blog images under
/content/dam/nzdoc/blogs/<upload year>, instead of paths derived from
the source URLs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="71">
   <si>
     <t>_reportFile</t>
   </si>
@@ -22,6 +22,9 @@
     <t>contentListMore</t>
   </si>
   <si>
+    <t>damImages</t>
+  </si>
+  <si>
     <t>heroImages</t>
   </si>
   <si>
@@ -52,7 +55,10 @@
     <t>Featured: https://www.doc.govt.nz/footer-links/new-on-the-site/; Media releases: https://www.doc.govt.nz/news/media-releases/2026-media-releases/</t>
   </si>
   <si>
-    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg</t>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg; https://www.doc.govt.nz/thumbs/gallery/contentassets/a8cf8502518043808b916575ca1bb512/denniston-hero.jpg -&gt; /content/dam/nzdoc/heros/denniston-hero.jpg; https://i0.wp.com/blog.doc.govt.nz/wp-content/uploads/2026/09/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg?w=200 -&gt; /content/dam/nzdoc/blogs/2026/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>index</t>
@@ -64,13 +70,160 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T02:52:36.786Z</t>
+    <t>2026-09-28T03:19:20.863Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
   </si>
   <si>
     <t>https://www.doc.govt.nz/</t>
+  </si>
+  <si>
+    <t>news/issues/bird-flu-updates.report.json</t>
+  </si>
+  <si>
+    <t>["breadcrumb","hero"]</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/globalassets/images/nature/native-animals/birds/brown-skua/brown-skua-1920.jpg -&gt; /content/dam/nzdoc/heros/brown-skua-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/issues/bird-flu-updates</t>
+  </si>
+  <si>
+    <t>article-hero</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:05:43.233Z</t>
+  </si>
+  <si>
+    <t>EMA: Bird flu updates: Issues</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/issues/bird-flu-updates/</t>
+  </si>
+  <si>
+    <t>about-us/our-role/managing-conservation/conservation-amendment-bill.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/59e382809add463ea8fa893707db334d/whakatane-hero.jpg -&gt; /content/dam/nzdoc/heros/whakatane-hero.jpg</t>
+  </si>
+  <si>
+    <t>about-us/our-role/managing-conservation/conservation-amendment-bill</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:05:57.831Z</t>
+  </si>
+  <si>
+    <t>EMA: Conservation Amendment Bill: Managing conservation</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/about-us/our-role/managing-conservation/conservation-amendment-bill/</t>
+  </si>
+  <si>
+    <t>news/events/national-events/national-wild-goat-hunting-competition.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/f7be0a20cbaa45f1b78b2d52b6d366b2/national-wild-goat-competition-2026-1920.jpg -&gt; /content/dam/nzdoc/heros/national-wild-goat-competition-2026-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/events/national-events/national-wild-goat-hunting-competition</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:14:05.267Z</t>
+  </si>
+  <si>
+    <t>EMA: National Wild Goat Hunting Competition 2026</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/events/national-events/national-wild-goat-hunting-competition/</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/6bd3432a1fe849b3848184b73ccc07b6/planting-with-damage-in-background1920.jpg -&gt; /content/dam/nzdoc/heros/planting-with-damage-in-background1920.jpg</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:06:25.267Z</t>
+  </si>
+  <si>
+    <t>EMA: 4WD group plants native trees to fix damage</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/media-releases/2026-media-releases/4wd-group-plants-native-trees-to-fix-damage/</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/funding-boost-for-bird-flu-surveillance.report.json</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/funding-boost-for-bird-flu-surveillance</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:06:12.822Z</t>
+  </si>
+  <si>
+    <t>EMA: Funding boost for bird flu surveillance: Media release 24 September 2026</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/media-releases/2026-media-releases/funding-boost-for-bird-flu-surveillance/</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/government-invests-in-cleaning-up-contaminated-crown-land.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/0e132745d3954aa8848ca8a263fb8400/puhipuhi-1920.jpg -&gt; /content/dam/nzdoc/heros/puhipuhi-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/government-invests-in-cleaning-up-contaminated-crown-land</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:06:18.888Z</t>
+  </si>
+  <si>
+    <t>EMA: Government invests in cleaning up contaminated Crown land: Media release 23 September 2026</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/media-releases/2026-media-releases/government-invests-in-cleaning-up-contaminated-crown-land/</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/toxoplasmosis-confirmed-as-cause-of-death-of-pregnant-hectors-dolphin.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/adba4374a3f54a75af306e54efe345f5/hectors-deceased-1920.jpg -&gt; /content/dam/nzdoc/heros/hectors-deceased-1920.jpg</t>
+  </si>
+  <si>
+    <t>news/media-releases/2026-media-releases/toxoplasmosis-confirmed-as-cause-of-death-of-pregnant-hectors-dolphin</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:06:32.869Z</t>
+  </si>
+  <si>
+    <t>EMA: Toxoplasmosis confirmed as cause of death of pregnant Hector’s dolphin: Media release 22 September 2026</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/news/media-releases/2026-media-releases/toxoplasmosis-confirmed-as-cause-of-death-of-pregnant-hectors-dolphin/</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/things-to-do/fishing/whitebaiting.report.json</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/thumbs/hero/contentassets/7844f904c74341bf9c8ddaefc05726ce/whitebaiter-in-westland-hero.jpg -&gt; /content/dam/nzdoc/heros/whitebaiter-in-westland-hero.jpg</t>
+  </si>
+  <si>
+    <t>parks-and-recreation/things-to-do/fishing/whitebaiting</t>
+  </si>
+  <si>
+    <t>2026-09-28T03:05:51.019Z</t>
+  </si>
+  <si>
+    <t>EMA: Whitebaiting: Things to do</t>
+  </si>
+  <si>
+    <t>https://www.doc.govt.nz/parks-and-recreation/things-to-do/fishing/whitebaiting/</t>
   </si>
 </sst>
 </file>
@@ -459,20 +612,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="19" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="4" width="50" customWidth="1"/>
-    <col min="5" max="5" width="7" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="26" customWidth="1"/>
-    <col min="9" max="9" width="33" customWidth="1"/>
-    <col min="10" max="10" width="26" customWidth="1"/>
+    <col min="3" max="6" width="50" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="11" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -503,41 +654,327 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" t="s">
         <v>17</v>
       </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" t="s">
-        <v>19</v>
+      <c r="H3" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J3" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+      <c r="G4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" t="s">
+        <v>38</v>
+      </c>
+      <c r="G5" t="s">
+        <v>17</v>
+      </c>
+      <c r="H5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>43</v>
+      </c>
+      <c r="F6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" t="s">
+        <v>26</v>
+      </c>
+      <c r="I6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" t="s">
+        <v>51</v>
+      </c>
+      <c r="K7" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>54</v>
+      </c>
+      <c r="F8" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" t="s">
+        <v>26</v>
+      </c>
+      <c r="I8" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" t="s">
+        <v>57</v>
+      </c>
+      <c r="K8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
+      <c r="J9" t="s">
+        <v>63</v>
+      </c>
+      <c r="K9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>66</v>
+      </c>
+      <c r="F10" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" t="s">
+        <v>69</v>
+      </c>
+      <c r="K10" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:K1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Reference homepage content lists to migrated articles
Import the Featured and Media releases lists as Content List blocks with
items mapped to /content/nzdoc page paths. Teasers read the image and
title from each referenced page's hero (subtitle from page metadata);
columns place the imported lists into their panels.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="69">
   <si>
     <t>_reportFile</t>
   </si>
@@ -19,9 +19,6 @@
     <t>blocks</t>
   </si>
   <si>
-    <t>contentListMore</t>
-  </si>
-  <si>
     <t>damImages</t>
   </si>
   <si>
@@ -52,9 +49,6 @@
     <t>["hero","cards","columns","feedback"]</t>
   </si>
   <si>
-    <t>Featured: https://www.doc.govt.nz/footer-links/new-on-the-site/; Media releases: https://www.doc.govt.nz/news/media-releases/2026-media-releases/</t>
-  </si>
-  <si>
     <t>https://www.doc.govt.nz/thumbs/hero/contentassets/9b48a55da5974906b6d65a89fb9d5d06/kura-tawhiti-hero.jpg -&gt; /content/dam/nzdoc/heros/kura-tawhiti-hero.jpg; https://www.doc.govt.nz/thumbs/gallery/contentassets/a8cf8502518043808b916575ca1bb512/denniston-hero.jpg -&gt; /content/dam/nzdoc/heros/denniston-hero.jpg; https://i0.wp.com/blog.doc.govt.nz/wp-content/uploads/2026/09/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg?w=200 -&gt; /content/dam/nzdoc/blogs/2026/black-robin-invertebrate-leon-everett-1-e1788825954346.jpg</t>
   </si>
   <si>
@@ -70,7 +64,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-09-28T03:19:20.863Z</t>
+    <t>2026-09-28T03:31:15.762Z</t>
   </si>
   <si>
     <t>EMA: Department of Conservation</t>
@@ -612,18 +606,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
     <col min="2" max="2" width="39" customWidth="1"/>
-    <col min="3" max="6" width="50" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="26" customWidth="1"/>
-    <col min="10" max="11" width="50" customWidth="1"/>
+    <col min="3" max="5" width="50" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -654,327 +648,297 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>10</v>
       </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J2" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="D3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="G3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" t="s">
+        <v>25</v>
+      </c>
+      <c r="I3" t="s">
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J4" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G5" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F6" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" t="s">
+        <v>43</v>
+      </c>
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="E7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F7" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" t="s">
+        <v>52</v>
+      </c>
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G8" t="s">
         <v>24</v>
       </c>
-      <c r="F3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I3" t="s">
-        <v>27</v>
-      </c>
-      <c r="J3" t="s">
-        <v>28</v>
-      </c>
-      <c r="K3" t="s">
-        <v>29</v>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" t="s">
+        <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" t="s">
+        <v>58</v>
+      </c>
+      <c r="E9" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="G9" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" t="s">
+        <v>60</v>
+      </c>
+      <c r="I9" t="s">
+        <v>61</v>
+      </c>
+      <c r="J9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E10" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>33</v>
-      </c>
-      <c r="J4" t="s">
-        <v>34</v>
-      </c>
-      <c r="K4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J5" t="s">
-        <v>40</v>
-      </c>
-      <c r="K5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>42</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G6" t="s">
-        <v>17</v>
-      </c>
-      <c r="H6" t="s">
-        <v>26</v>
-      </c>
-      <c r="I6" t="s">
-        <v>45</v>
-      </c>
-      <c r="J6" t="s">
-        <v>46</v>
-      </c>
-      <c r="K6" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="G10" t="s">
         <v>24</v>
       </c>
-      <c r="F7" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" t="s">
-        <v>17</v>
-      </c>
-      <c r="H7" t="s">
-        <v>26</v>
-      </c>
-      <c r="I7" t="s">
-        <v>50</v>
-      </c>
-      <c r="J7" t="s">
-        <v>51</v>
-      </c>
-      <c r="K7" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" t="s">
-        <v>26</v>
-      </c>
-      <c r="I8" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" t="s">
-        <v>57</v>
-      </c>
-      <c r="K8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" t="s">
-        <v>62</v>
-      </c>
-      <c r="J9" t="s">
-        <v>63</v>
-      </c>
-      <c r="K9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="H10" t="s">
         <v>66</v>
       </c>
-      <c r="F10" t="s">
+      <c r="I10" t="s">
         <v>67</v>
       </c>
-      <c r="G10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>68</v>
-      </c>
-      <c r="J10" t="s">
-        <v>69</v>
-      </c>
-      <c r="K10" t="s">
-        <v>70</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>